<commit_message>
modified the config file
</commit_message>
<xml_diff>
--- a/config/kabelconfig_duitslandlaan.xlsx
+++ b/config/kabelconfig_duitslandlaan.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-135" yWindow="-135" windowWidth="77070" windowHeight="21150" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="77040" windowHeight="21120" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="0_Parameters" sheetId="1" state="visible" r:id="rId1"/>
@@ -75,7 +75,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -90,6 +90,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -131,13 +137,13 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="6" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="left"/>
       <protection locked="0" hidden="0"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -507,10 +513,10 @@
   <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" style="9" min="1" max="1"/>
-    <col width="18" customWidth="1" style="9" min="2" max="2"/>
-    <col width="30" customWidth="1" style="9" min="3" max="3"/>
-    <col width="74" customWidth="1" style="9" min="4" max="4"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="74" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -544,79 +550,79 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>project_nr</t>
         </is>
       </c>
-      <c r="B4" s="7" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>PR 20267283-2600206</t>
         </is>
       </c>
-      <c r="C4" s="7" t="n"/>
-      <c r="D4" s="7" t="inlineStr">
+      <c r="C4" s="3" t="n"/>
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>Erco PR number</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>project_naam</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>Duitslandlaan Zoetermeer</t>
         </is>
       </c>
-      <c r="C5" s="7" t="n"/>
-      <c r="D5" s="7" t="n"/>
+      <c r="C5" s="3" t="n"/>
+      <c r="D5" s="3" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>rk_naam</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>RK071</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>AUTO or fixed (e.g. RK071)</t>
         </is>
       </c>
-      <c r="D6" s="7" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>AUTO = derived from the process-code prefixes</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>plaats_rk</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Technische ruimte begane grond</t>
         </is>
       </c>
-      <c r="C7" s="7" t="n"/>
-      <c r="D7" s="7" t="inlineStr">
+      <c r="C7" s="3" t="n"/>
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>human input, NOT present in the I/O list</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>brandklasse</t>
         </is>
@@ -626,19 +632,19 @@
           <t>B2CA</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>CCA / B2CA</t>
         </is>
       </c>
-      <c r="D8" s="7" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>MANDATORY — not derivable from the I/O list (Duitslandlaan + 112-meldkamer lesson)</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>signaalfamilie</t>
         </is>
@@ -648,96 +654,96 @@
           <t>JOBA</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>DRAK / JOBA</t>
         </is>
       </c>
-      <c r="D9" s="7" t="inlineStr">
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>CCA -&gt; usually DRAK, B2CA -&gt; usually JOBA; confirm per project</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="inlineStr">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>lengteklasse</t>
         </is>
       </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>&lt;=50m</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>&lt;=50m / 50-100m</t>
         </is>
       </c>
-      <c r="D10" s="7" t="inlineStr">
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>&gt;50m -&gt; JOBA variant + 'max ..m' note</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>naregelsysteem</t>
         </is>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>geen</t>
         </is>
       </c>
-      <c r="C11" s="7" t="inlineStr">
+      <c r="C11" s="3" t="inlineStr">
         <is>
           <t>geen / BRN15 / Priva / Touchpoint</t>
         </is>
       </c>
-      <c r="D11" s="7" t="inlineStr">
+      <c r="D11" s="3" t="inlineStr">
         <is>
           <t>determines the bus cable + room-control item set</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="inlineStr">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>tracing_scope</t>
         </is>
       </c>
-      <c r="B12" s="7" t="inlineStr">
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>erco</t>
         </is>
       </c>
-      <c r="C12" s="7" t="inlineStr">
+      <c r="C12" s="3" t="inlineStr">
         <is>
           <t>erco / derden</t>
         </is>
       </c>
-      <c r="D12" s="7" t="inlineStr">
+      <c r="D12" s="3" t="inlineStr">
         <is>
           <t>Duitslandlaan precedent: Erco feeds from the RK, despite the input remark</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="inlineStr">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>locatie_veld_standaard</t>
         </is>
       </c>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>in TR</t>
         </is>
       </c>
-      <c r="C13" s="7" t="n"/>
-      <c r="D13" s="7" t="inlineStr">
+      <c r="C13" s="3" t="n"/>
+      <c r="D13" s="3" t="inlineStr">
         <is>
           <t>default 'bekabeling naar' for field cables</t>
         </is>
@@ -820,13 +826,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D122"/>
+  <dimension ref="A1:D141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="36" customWidth="1" style="9" min="1" max="1"/>
-    <col width="24" customWidth="1" style="9" min="2" max="2"/>
-    <col width="10" customWidth="1" style="9" min="3" max="3"/>
-    <col width="62" customWidth="1" style="9" min="4" max="4"/>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="62" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -859,988 +865,988 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>modbus ip</t>
         </is>
       </c>
-      <c r="B4" s="7" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>BUS_MODBUS</t>
         </is>
       </c>
-      <c r="C4" s="7" t="n">
+      <c r="C4" s="3" t="n">
         <v>90</v>
       </c>
-      <c r="D4" s="7" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>Duitslandlaan AIR-SEP: Modbus-IP field device -&gt; BMS cable</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>modbus</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>BUS_MODBUS</t>
         </is>
       </c>
-      <c r="C5" s="7" t="n">
+      <c r="C5" s="3" t="n">
         <v>50</v>
       </c>
-      <c r="D5" s="7" t="n"/>
+      <c r="D5" s="3" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>bacnet ms/tp</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>BUS_MODBUS</t>
         </is>
       </c>
-      <c r="C6" s="7" t="n">
+      <c r="C6" s="3" t="n">
         <v>60</v>
       </c>
-      <c r="D6" s="7" t="n"/>
+      <c r="D6" s="3" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>bacnet</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>BUS_IP_PANEEL</t>
         </is>
       </c>
-      <c r="C7" s="7" t="n">
+      <c r="C7" s="3" t="n">
         <v>55</v>
       </c>
-      <c r="D7" s="7" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>112: BACnet/IP -&gt; COMM CAT6, per device, no daisy-chain</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>m-bus</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>BUS_MBUS</t>
         </is>
       </c>
-      <c r="C8" s="7" t="n">
+      <c r="C8" s="3" t="n">
         <v>60</v>
       </c>
-      <c r="D8" s="7" t="n"/>
+      <c r="D8" s="3" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>buskoppeling</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>BUS_MODBUS</t>
         </is>
       </c>
-      <c r="C9" s="7" t="n">
+      <c r="C9" s="3" t="n">
         <v>40</v>
       </c>
-      <c r="D9" s="7" t="n"/>
+      <c r="D9" s="3" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="inlineStr">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>mod-bus</t>
         </is>
       </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>BUS_MODBUS</t>
         </is>
       </c>
-      <c r="C10" s="7" t="n">
+      <c r="C10" s="3" t="n">
         <v>60</v>
       </c>
-      <c r="D10" s="7" t="n"/>
+      <c r="D10" s="3" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>communicatie interface</t>
         </is>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>BUS_INTERFACE</t>
         </is>
       </c>
-      <c r="C11" s="7" t="n">
+      <c r="C11" s="3" t="n">
         <v>70</v>
       </c>
-      <c r="D11" s="7" t="inlineStr">
+      <c r="D11" s="3" t="inlineStr">
         <is>
           <t>CIM200 print: belongs to the pump, generates no cable of its own</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="inlineStr">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>touchpanel</t>
         </is>
       </c>
-      <c r="B12" s="7" t="inlineStr">
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>BUS_IP_PANEEL</t>
         </is>
       </c>
-      <c r="C12" s="7" t="n">
+      <c r="C12" s="3" t="n">
         <v>70</v>
       </c>
-      <c r="D12" s="7" t="n"/>
+      <c r="D12" s="3" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="inlineStr">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>kwh-meter</t>
         </is>
       </c>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>ENERGIEMETER</t>
         </is>
       </c>
-      <c r="C13" s="7" t="n">
+      <c r="C13" s="3" t="n">
         <v>60</v>
       </c>
-      <c r="D13" s="7" t="n"/>
+      <c r="D13" s="3" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="inlineStr">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>energiemeter</t>
         </is>
       </c>
-      <c r="B14" s="7" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
         <is>
           <t>ENERGIEMETER</t>
         </is>
       </c>
-      <c r="C14" s="7" t="n">
+      <c r="C14" s="3" t="n">
         <v>60</v>
       </c>
-      <c r="D14" s="7" t="inlineStr">
+      <c r="D14" s="3" t="inlineStr">
         <is>
           <t>RH33: bus + separate 24V feed cable</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="inlineStr">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>koudemeter</t>
         </is>
       </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>ENERGIEMETER</t>
         </is>
       </c>
-      <c r="C15" s="7" t="n">
+      <c r="C15" s="3" t="n">
         <v>60</v>
       </c>
-      <c r="D15" s="7" t="n"/>
+      <c r="D15" s="3" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="7" t="inlineStr">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>warmtemeter</t>
         </is>
       </c>
-      <c r="B16" s="7" t="inlineStr">
+      <c r="B16" s="3" t="inlineStr">
         <is>
           <t>ENERGIEMETER</t>
         </is>
       </c>
-      <c r="C16" s="7" t="n">
+      <c r="C16" s="3" t="n">
         <v>60</v>
       </c>
-      <c r="D16" s="7" t="n"/>
+      <c r="D16" s="3" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="7" t="inlineStr">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>flowmeting</t>
         </is>
       </c>
-      <c r="B17" s="7" t="inlineStr">
+      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>METING_ACTIEF</t>
         </is>
       </c>
-      <c r="C17" s="7" t="n">
+      <c r="C17" s="3" t="n">
         <v>70</v>
       </c>
-      <c r="D17" s="7" t="inlineStr">
+      <c r="D17" s="3" t="inlineStr">
         <is>
           <t>prio raised above energiemeter tie</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="7" t="inlineStr">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>flowmeter</t>
         </is>
       </c>
-      <c r="B18" s="7" t="inlineStr">
+      <c r="B18" s="3" t="inlineStr">
         <is>
           <t>METING_ACTIEF</t>
         </is>
       </c>
-      <c r="C18" s="7" t="n">
+      <c r="C18" s="3" t="n">
         <v>70</v>
       </c>
-      <c r="D18" s="7" t="n"/>
+      <c r="D18" s="3" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="7" t="inlineStr">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>optie c1</t>
         </is>
       </c>
-      <c r="B19" s="7" t="inlineStr">
+      <c r="B19" s="3" t="inlineStr">
         <is>
           <t>METER_OPTIE_VOELER</t>
         </is>
       </c>
-      <c r="C19" s="7" t="n">
+      <c r="C19" s="3" t="n">
         <v>90</v>
       </c>
-      <c r="D19" s="7" t="inlineStr">
+      <c r="D19" s="3" t="inlineStr">
         <is>
           <t>PT100 of an E+H meter -&gt; 'Via aansluitsnoer', no cable</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="7" t="inlineStr">
+      <c r="A20" s="3" t="inlineStr">
         <is>
           <t>pt100</t>
         </is>
       </c>
-      <c r="B20" s="7" t="inlineStr">
+      <c r="B20" s="3" t="inlineStr">
         <is>
           <t>METER_OPTIE_VOELER</t>
         </is>
       </c>
-      <c r="C20" s="7" t="n">
+      <c r="C20" s="3" t="n">
         <v>40</v>
       </c>
-      <c r="D20" s="7" t="inlineStr">
+      <c r="D20" s="3" t="inlineStr">
         <is>
           <t>only when tied to an energy meter; otherwise METING_PASSIEF</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="7" t="inlineStr">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t>drukverschil</t>
         </is>
       </c>
-      <c r="B21" s="7" t="inlineStr">
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t>METING_ACTIEF</t>
         </is>
       </c>
-      <c r="C21" s="7" t="n">
+      <c r="C21" s="3" t="n">
         <v>60</v>
       </c>
-      <c r="D21" s="7" t="inlineStr">
+      <c r="D21" s="3" t="inlineStr">
         <is>
           <t>22WDP -&gt; 5X1/2502Q</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="7" t="inlineStr">
+      <c r="A22" s="3" t="inlineStr">
         <is>
           <t>systeemdruk</t>
         </is>
       </c>
-      <c r="B22" s="7" t="inlineStr">
+      <c r="B22" s="3" t="inlineStr">
         <is>
           <t>METING_ACTIEF</t>
         </is>
       </c>
-      <c r="C22" s="7" t="n">
+      <c r="C22" s="3" t="n">
         <v>60</v>
       </c>
-      <c r="D22" s="7" t="inlineStr">
+      <c r="D22" s="3" t="inlineStr">
         <is>
           <t>22WP-119</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="7" t="inlineStr">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>druk</t>
         </is>
       </c>
-      <c r="B23" s="7" t="inlineStr">
+      <c r="B23" s="3" t="inlineStr">
         <is>
           <t>METING_ACTIEF</t>
         </is>
       </c>
-      <c r="C23" s="7" t="n">
+      <c r="C23" s="3" t="n">
         <v>30</v>
       </c>
-      <c r="D23" s="7" t="n"/>
+      <c r="D23" s="3" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="7" t="inlineStr">
+      <c r="A24" s="3" t="inlineStr">
         <is>
           <t>temperatuur</t>
         </is>
       </c>
-      <c r="B24" s="7" t="inlineStr">
+      <c r="B24" s="3" t="inlineStr">
         <is>
           <t>METING_PASSIEF</t>
         </is>
       </c>
-      <c r="C24" s="7" t="n">
+      <c r="C24" s="3" t="n">
         <v>65</v>
       </c>
-      <c r="D24" s="7" t="inlineStr">
+      <c r="D24" s="3" t="inlineStr">
         <is>
           <t>prio raised above warmtepomp(40) — Boerhaave over-match fix</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="7" t="inlineStr">
+      <c r="A25" s="3" t="inlineStr">
         <is>
           <t>buitenvoeler</t>
         </is>
       </c>
-      <c r="B25" s="7" t="inlineStr">
+      <c r="B25" s="3" t="inlineStr">
         <is>
           <t>METING_ACTIEF</t>
         </is>
       </c>
-      <c r="C25" s="7" t="n">
+      <c r="C25" s="3" t="n">
         <v>60</v>
       </c>
-      <c r="D25" s="7" t="inlineStr">
+      <c r="D25" s="3" t="inlineStr">
         <is>
           <t>only if present in the input (lesson: do not add it yourself)</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="7" t="inlineStr">
+      <c r="A26" s="3" t="inlineStr">
         <is>
           <t>blokkeerafsluiter</t>
         </is>
       </c>
-      <c r="B26" s="7" t="inlineStr">
+      <c r="B26" s="3" t="inlineStr">
         <is>
           <t>KLEP_STURING_MELDING</t>
         </is>
       </c>
-      <c r="C26" s="7" t="n">
+      <c r="C26" s="3" t="n">
         <v>70</v>
       </c>
-      <c r="D26" s="7" t="inlineStr">
+      <c r="D26" s="3" t="inlineStr">
         <is>
           <t>GR24A-SR: control + feedback -&gt; 7X1</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="7" t="inlineStr">
+      <c r="A27" s="3" t="inlineStr">
         <is>
           <t>regelafsluiter open/dicht</t>
         </is>
       </c>
-      <c r="B27" s="7" t="inlineStr">
+      <c r="B27" s="3" t="inlineStr">
         <is>
           <t>KLEP_STURING_MELDING</t>
         </is>
       </c>
-      <c r="C27" s="7" t="n">
+      <c r="C27" s="3" t="n">
         <v>80</v>
       </c>
-      <c r="D27" s="7" t="n"/>
+      <c r="D27" s="3" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="7" t="inlineStr">
+      <c r="A28" s="3" t="inlineStr">
         <is>
           <t>regelafsluiter</t>
         </is>
       </c>
-      <c r="B28" s="7" t="inlineStr">
+      <c r="B28" s="3" t="inlineStr">
         <is>
           <t>REGELAFSLUITER_0_10V</t>
         </is>
       </c>
-      <c r="C28" s="7" t="n">
+      <c r="C28" s="3" t="n">
         <v>50</v>
       </c>
-      <c r="D28" s="7" t="inlineStr">
+      <c r="D28" s="3" t="inlineStr">
         <is>
           <t>0-10V -&gt; 5X1 / RAK 4X0,8</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="7" t="inlineStr">
+      <c r="A29" s="3" t="inlineStr">
         <is>
           <t>klep</t>
         </is>
       </c>
-      <c r="B29" s="7" t="inlineStr">
+      <c r="B29" s="3" t="inlineStr">
         <is>
           <t>KLEP_OD</t>
         </is>
       </c>
-      <c r="C29" s="7" t="n">
+      <c r="C29" s="3" t="n">
         <v>30</v>
       </c>
-      <c r="D29" s="7" t="n"/>
+      <c r="D29" s="3" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="7" t="inlineStr">
+      <c r="A30" s="3" t="inlineStr">
         <is>
           <t>brandklep</t>
         </is>
       </c>
-      <c r="B30" s="7" t="inlineStr">
+      <c r="B30" s="3" t="inlineStr">
         <is>
           <t>BRANDKLEP</t>
         </is>
       </c>
-      <c r="C30" s="7" t="n">
+      <c r="C30" s="3" t="n">
         <v>70</v>
       </c>
-      <c r="D30" s="7" t="inlineStr">
+      <c r="D30" s="3" t="inlineStr">
         <is>
           <t>112: one 2-core cable PER damper, do not bundle</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="7" t="inlineStr">
+      <c r="A31" s="3" t="inlineStr">
         <is>
           <t>vrijgave</t>
         </is>
       </c>
-      <c r="B31" s="7" t="inlineStr">
+      <c r="B31" s="3" t="inlineStr">
         <is>
           <t>VRIJGAVE</t>
         </is>
       </c>
-      <c r="C31" s="7" t="n">
+      <c r="C31" s="3" t="n">
         <v>50</v>
       </c>
-      <c r="D31" s="7" t="n"/>
+      <c r="D31" s="3" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="7" t="inlineStr">
+      <c r="A32" s="3" t="inlineStr">
         <is>
           <t>sturing 0-10</t>
         </is>
       </c>
-      <c r="B32" s="7" t="inlineStr">
+      <c r="B32" s="3" t="inlineStr">
         <is>
           <t>STURING_0_10V</t>
         </is>
       </c>
-      <c r="C32" s="7" t="n">
+      <c r="C32" s="3" t="n">
         <v>60</v>
       </c>
-      <c r="D32" s="7" t="n"/>
+      <c r="D32" s="3" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="7" t="inlineStr">
+      <c r="A33" s="3" t="inlineStr">
         <is>
           <t>sturing</t>
         </is>
       </c>
-      <c r="B33" s="7" t="inlineStr">
+      <c r="B33" s="3" t="inlineStr">
         <is>
           <t>STURING_0_10V</t>
         </is>
       </c>
-      <c r="C33" s="7" t="n">
+      <c r="C33" s="3" t="n">
         <v>30</v>
       </c>
-      <c r="D33" s="7" t="inlineStr">
+      <c r="D33" s="3" t="inlineStr">
         <is>
           <t>E-boiler: AO on its own 2-core cable</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="7" t="inlineStr">
+      <c r="A34" s="3" t="inlineStr">
         <is>
           <t>bedrijf/storing</t>
         </is>
       </c>
-      <c r="B34" s="7" t="inlineStr">
+      <c r="B34" s="3" t="inlineStr">
         <is>
           <t>BEDRIJF_STORING</t>
         </is>
       </c>
-      <c r="C34" s="7" t="n">
+      <c r="C34" s="3" t="n">
         <v>60</v>
       </c>
-      <c r="D34" s="7" t="n"/>
+      <c r="D34" s="3" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="7" t="inlineStr">
+      <c r="A35" s="3" t="inlineStr">
         <is>
           <t>bedrijfsmeldingen</t>
         </is>
       </c>
-      <c r="B35" s="7" t="inlineStr">
+      <c r="B35" s="3" t="inlineStr">
         <is>
           <t>MELDINGEN_GROOT</t>
         </is>
       </c>
-      <c r="C35" s="7" t="n">
+      <c r="C35" s="3" t="n">
         <v>70</v>
       </c>
-      <c r="D35" s="7" t="inlineStr">
+      <c r="D35" s="3" t="inlineStr">
         <is>
           <t>WP: all meldingen on one 12X1</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="7" t="inlineStr">
+      <c r="A36" s="3" t="inlineStr">
         <is>
           <t>diverse meldingen</t>
         </is>
       </c>
-      <c r="B36" s="7" t="inlineStr">
+      <c r="B36" s="3" t="inlineStr">
         <is>
           <t>MELDINGEN_GROOT</t>
         </is>
       </c>
-      <c r="C36" s="7" t="n">
+      <c r="C36" s="3" t="n">
         <v>70</v>
       </c>
-      <c r="D36" s="7" t="n"/>
+      <c r="D36" s="3" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="7" t="inlineStr">
+      <c r="A37" s="3" t="inlineStr">
         <is>
           <t>storing</t>
         </is>
       </c>
-      <c r="B37" s="7" t="inlineStr">
+      <c r="B37" s="3" t="inlineStr">
         <is>
           <t>MELDING</t>
         </is>
       </c>
-      <c r="C37" s="7" t="n">
+      <c r="C37" s="3" t="n">
         <v>30</v>
       </c>
-      <c r="D37" s="7" t="inlineStr">
+      <c r="D37" s="3" t="inlineStr">
         <is>
           <t>single contact -&gt; 2X1/2X0,8</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="7" t="inlineStr">
+      <c r="A38" s="3" t="inlineStr">
         <is>
           <t>melding</t>
         </is>
       </c>
-      <c r="B38" s="7" t="inlineStr">
+      <c r="B38" s="3" t="inlineStr">
         <is>
           <t>MELDING</t>
         </is>
       </c>
-      <c r="C38" s="7" t="n">
+      <c r="C38" s="3" t="n">
         <v>25</v>
       </c>
-      <c r="D38" s="7" t="n"/>
+      <c r="D38" s="3" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="7" t="inlineStr">
+      <c r="A39" s="3" t="inlineStr">
         <is>
           <t>tracing</t>
         </is>
       </c>
-      <c r="B39" s="7" t="inlineStr">
+      <c r="B39" s="3" t="inlineStr">
         <is>
           <t>TRACING</t>
         </is>
       </c>
-      <c r="C39" s="7" t="n">
+      <c r="C39" s="3" t="n">
         <v>70</v>
       </c>
-      <c r="D39" s="7" t="inlineStr">
+      <c r="D39" s="3" t="inlineStr">
         <is>
           <t>feed from the RK (ws=1) + 2-core feedback</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="7" t="inlineStr">
+      <c r="A40" s="3" t="inlineStr">
         <is>
           <t>warmtepomp</t>
         </is>
       </c>
-      <c r="B40" s="7" t="inlineStr">
+      <c r="B40" s="3" t="inlineStr">
         <is>
           <t>WARMTEPOMP</t>
         </is>
       </c>
-      <c r="C40" s="7" t="n">
+      <c r="C40" s="3" t="n">
         <v>40</v>
       </c>
-      <c r="D40" s="7" t="inlineStr">
+      <c r="D40" s="3" t="inlineStr">
         <is>
           <t>bus + meldingen bundle; feed = Werkzaamheden derden</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="7" t="inlineStr">
+      <c r="A41" s="3" t="inlineStr">
         <is>
           <t>elektrische ketel</t>
         </is>
       </c>
-      <c r="B41" s="7" t="inlineStr">
+      <c r="B41" s="3" t="inlineStr">
         <is>
           <t>E_KETEL</t>
         </is>
       </c>
-      <c r="C41" s="7" t="n">
+      <c r="C41" s="3" t="n">
         <v>70</v>
       </c>
-      <c r="D41" s="7" t="inlineStr">
+      <c r="D41" s="3" t="inlineStr">
         <is>
           <t>vrijgave/storing 5X1 + separate sturing 2X1; feed by third parties</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="7" t="inlineStr">
+      <c r="A42" s="3" t="inlineStr">
         <is>
           <t>levering derden</t>
         </is>
       </c>
-      <c r="B42" s="7" t="inlineStr">
+      <c r="B42" s="3" t="inlineStr">
         <is>
           <t>DERDEN</t>
         </is>
       </c>
-      <c r="C42" s="7" t="n">
+      <c r="C42" s="3" t="n">
         <v>80</v>
       </c>
-      <c r="D42" s="7" t="n"/>
+      <c r="D42" s="3" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="7" t="inlineStr">
+      <c r="A43" s="3" t="inlineStr">
         <is>
           <t>levering derde</t>
         </is>
       </c>
-      <c r="B43" s="7" t="inlineStr">
+      <c r="B43" s="3" t="inlineStr">
         <is>
           <t>DERDEN</t>
         </is>
       </c>
-      <c r="C43" s="7" t="n">
+      <c r="C43" s="3" t="n">
         <v>80</v>
       </c>
-      <c r="D43" s="7" t="n"/>
+      <c r="D43" s="3" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="7" t="inlineStr">
+      <c r="A44" s="3" t="inlineStr">
         <is>
           <t>vanuit bmc</t>
         </is>
       </c>
-      <c r="B44" s="7" t="inlineStr">
+      <c r="B44" s="3" t="inlineStr">
         <is>
           <t>DERDEN</t>
         </is>
       </c>
-      <c r="C44" s="7" t="n">
+      <c r="C44" s="3" t="n">
         <v>80</v>
       </c>
-      <c r="D44" s="7" t="n"/>
+      <c r="D44" s="3" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="7" t="inlineStr">
+      <c r="A45" s="3" t="inlineStr">
         <is>
           <t>uit e-installatie</t>
         </is>
       </c>
-      <c r="B45" s="7" t="inlineStr">
+      <c r="B45" s="3" t="inlineStr">
         <is>
           <t>DERDEN</t>
         </is>
       </c>
-      <c r="C45" s="7" t="n">
+      <c r="C45" s="3" t="n">
         <v>80</v>
       </c>
-      <c r="D45" s="7" t="n"/>
+      <c r="D45" s="3" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="7" t="inlineStr">
+      <c r="A46" s="3" t="inlineStr">
         <is>
           <t>vanuit e-verdeler</t>
         </is>
       </c>
-      <c r="B46" s="7" t="inlineStr">
+      <c r="B46" s="3" t="inlineStr">
         <is>
           <t>DERDEN</t>
         </is>
       </c>
-      <c r="C46" s="7" t="n">
+      <c r="C46" s="3" t="n">
         <v>80</v>
       </c>
-      <c r="D46" s="7" t="n"/>
+      <c r="D46" s="3" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="7" t="inlineStr">
+      <c r="A47" s="3" t="inlineStr">
         <is>
           <t>vanuit hvk</t>
         </is>
       </c>
-      <c r="B47" s="7" t="inlineStr">
+      <c r="B47" s="3" t="inlineStr">
         <is>
           <t>DERDEN</t>
         </is>
       </c>
-      <c r="C47" s="7" t="n">
+      <c r="C47" s="3" t="n">
         <v>80</v>
       </c>
-      <c r="D47" s="7" t="n"/>
+      <c r="D47" s="3" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="7" t="inlineStr">
+      <c r="A48" s="3" t="inlineStr">
         <is>
           <t>voeding door derden</t>
         </is>
       </c>
-      <c r="B48" s="7" t="inlineStr">
+      <c r="B48" s="3" t="inlineStr">
         <is>
           <t>DERDEN</t>
         </is>
       </c>
-      <c r="C48" s="7" t="n">
+      <c r="C48" s="3" t="n">
         <v>85</v>
       </c>
-      <c r="D48" s="7" t="n"/>
+      <c r="D48" s="3" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="7" t="inlineStr">
+      <c r="A49" s="3" t="inlineStr">
         <is>
           <t>regelkast</t>
         </is>
       </c>
-      <c r="B49" s="7" t="inlineStr">
+      <c r="B49" s="3" t="inlineStr">
         <is>
           <t>REGELKAST</t>
         </is>
       </c>
-      <c r="C49" s="7" t="n">
+      <c r="C49" s="3" t="n">
         <v>90</v>
       </c>
-      <c r="D49" s="7" t="inlineStr">
+      <c r="D49" s="3" t="inlineStr">
         <is>
           <t>own feed = Kabel levering derde totaan RK</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="7" t="inlineStr">
+      <c r="A50" s="3" t="inlineStr">
         <is>
           <t>n.t.b.</t>
         </is>
       </c>
-      <c r="B50" s="7" t="inlineStr">
+      <c r="B50" s="3" t="inlineStr">
         <is>
           <t>NTB</t>
         </is>
       </c>
-      <c r="C50" s="7" t="n">
+      <c r="C50" s="3" t="n">
         <v>85</v>
       </c>
-      <c r="D50" s="7" t="inlineStr">
+      <c r="D50" s="3" t="inlineStr">
         <is>
           <t>unknown scope -&gt; omit + flag</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="7" t="inlineStr">
+      <c r="A51" s="3" t="inlineStr">
         <is>
           <t>brandmelding</t>
         </is>
       </c>
-      <c r="B51" s="7" t="inlineStr">
+      <c r="B51" s="3" t="inlineStr">
         <is>
           <t>BRANDMELDING</t>
         </is>
       </c>
-      <c r="C51" s="7" t="n">
+      <c r="C51" s="3" t="n">
         <v>80</v>
       </c>
-      <c r="D51" s="7" t="inlineStr">
+      <c r="D51" s="3" t="inlineStr">
         <is>
           <t>always present in Onderstation algemeen</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="7" t="inlineStr">
+      <c r="A52" s="3" t="inlineStr">
         <is>
           <t>circulatiepomp</t>
         </is>
       </c>
-      <c r="B52" s="7" t="inlineStr">
+      <c r="B52" s="3" t="inlineStr">
         <is>
           <t>POMP</t>
         </is>
       </c>
-      <c r="C52" s="7" t="n">
+      <c r="C52" s="3" t="n">
         <v>50</v>
       </c>
-      <c r="D52" s="7" t="n"/>
+      <c r="D52" s="3" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" s="7" t="inlineStr">
+      <c r="A53" s="3" t="inlineStr">
         <is>
           <t>circulaite pomp</t>
         </is>
       </c>
-      <c r="B53" s="7" t="inlineStr">
+      <c r="B53" s="3" t="inlineStr">
         <is>
           <t>POMP</t>
         </is>
       </c>
-      <c r="C53" s="7" t="n">
+      <c r="C53" s="3" t="n">
         <v>50</v>
       </c>
-      <c r="D53" s="7" t="inlineStr">
+      <c r="D53" s="3" t="inlineStr">
         <is>
           <t>typo variant seen in the input</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="7" t="inlineStr">
+      <c r="A54" s="3" t="inlineStr">
         <is>
           <t>circ.pomp</t>
         </is>
       </c>
-      <c r="B54" s="7" t="inlineStr">
+      <c r="B54" s="3" t="inlineStr">
         <is>
           <t>POMP</t>
         </is>
       </c>
-      <c r="C54" s="7" t="n">
+      <c r="C54" s="3" t="n">
         <v>50</v>
       </c>
-      <c r="D54" s="7" t="n"/>
+      <c r="D54" s="3" t="n"/>
     </row>
     <row r="55">
-      <c r="A55" s="7" t="inlineStr">
+      <c r="A55" s="3" t="inlineStr">
         <is>
           <t>transportpomp</t>
         </is>
       </c>
-      <c r="B55" s="7" t="inlineStr">
+      <c r="B55" s="3" t="inlineStr">
         <is>
           <t>POMP</t>
         </is>
       </c>
-      <c r="C55" s="7" t="n">
+      <c r="C55" s="3" t="n">
         <v>50</v>
       </c>
-      <c r="D55" s="7" t="inlineStr">
+      <c r="D55" s="3" t="inlineStr">
         <is>
           <t>400V without N -&gt; 4G2,5 (NOT 5G)</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="7" t="inlineStr">
+      <c r="A56" s="3" t="inlineStr">
         <is>
           <t>pomp</t>
         </is>
       </c>
-      <c r="B56" s="7" t="inlineStr">
+      <c r="B56" s="3" t="inlineStr">
         <is>
           <t>POMP</t>
         </is>
       </c>
-      <c r="C56" s="7" t="n">
+      <c r="C56" s="3" t="n">
         <v>25</v>
       </c>
-      <c r="D56" s="7" t="n"/>
+      <c r="D56" s="3" t="n"/>
     </row>
     <row r="57">
-      <c r="A57" s="7" t="inlineStr">
+      <c r="A57" s="3" t="inlineStr">
         <is>
           <t>ontgasser</t>
         </is>
       </c>
-      <c r="B57" s="7" t="inlineStr">
+      <c r="B57" s="3" t="inlineStr">
         <is>
           <t>APPARAAT_230V</t>
         </is>
       </c>
-      <c r="C57" s="7" t="n">
+      <c r="C57" s="3" t="n">
         <v>50</v>
       </c>
-      <c r="D57" s="7" t="inlineStr">
+      <c r="D57" s="3" t="inlineStr">
         <is>
           <t>Korex AIR-SEP: feed + fault + bus</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="7" t="inlineStr">
+      <c r="A58" s="3" t="inlineStr">
         <is>
           <t>ventilator</t>
         </is>
       </c>
-      <c r="B58" s="7" t="inlineStr">
+      <c r="B58" s="3" t="inlineStr">
         <is>
           <t>EC_VENTILATOR</t>
         </is>
       </c>
-      <c r="C58" s="7" t="n">
+      <c r="C58" s="3" t="n">
         <v>40</v>
       </c>
-      <c r="D58" s="7" t="inlineStr">
+      <c r="D58" s="3" t="inlineStr">
         <is>
           <t>run/fault/control -&gt; 3X2 AFG</t>
         </is>
@@ -3104,6 +3110,360 @@
         <is>
           <t xml:space="preserve">	same, matched on omschrijving (OCR-safe alternative)</t>
         </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>resetknop</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>PANEL_INTERN</t>
+        </is>
+      </c>
+      <c r="C123" t="n">
+        <v>85</v>
+      </c>
+      <c r="D123" t="n">
+        <v>7267</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>reset storingen</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>PANEL_INTERN</t>
+        </is>
+      </c>
+      <c r="C124" t="n">
+        <v>85</v>
+      </c>
+      <c r="D124" s="9" t="inlineStr">
+        <is>
+          <t>2195-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>reset drukknop</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>PANEL_INTERN</t>
+        </is>
+      </c>
+      <c r="C125" t="n">
+        <v>85</v>
+      </c>
+      <c r="D125" s="9" t="inlineStr">
+        <is>
+          <t>2195-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>installatie automaten</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>PANEL_INTERN</t>
+        </is>
+      </c>
+      <c r="C126" t="n">
+        <v>85</v>
+      </c>
+      <c r="D126" s="9" t="inlineStr">
+        <is>
+          <t>2195-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>automaat 230V</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>PANEL_INTERN</t>
+        </is>
+      </c>
+      <c r="C127" t="n">
+        <v>85</v>
+      </c>
+      <c r="D127" s="9" t="inlineStr">
+        <is>
+          <t>7267</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>automaat 24V</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>PANEL_INTERN</t>
+        </is>
+      </c>
+      <c r="C128" t="n">
+        <v>85</v>
+      </c>
+      <c r="D128" s="9" t="inlineStr">
+        <is>
+          <t>7267</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>netwatcher</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>PANEL_INTERN</t>
+        </is>
+      </c>
+      <c r="C129" t="n">
+        <v>85</v>
+      </c>
+      <c r="D129" s="9" t="inlineStr">
+        <is>
+          <t>2195-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>afsluiter</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>KLEP_OD</t>
+        </is>
+      </c>
+      <c r="C130" t="n">
+        <v>20</v>
+      </c>
+      <c r="D130" t="n">
+        <v>7222</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>kogelafsluiter</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>KLEP_OD</t>
+        </is>
+      </c>
+      <c r="C131" t="n">
+        <v>40</v>
+      </c>
+      <c r="D131" t="n">
+        <v>7222</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>priva blue id</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>PANEL_INTERN</t>
+        </is>
+      </c>
+      <c r="C132" t="n">
+        <v>85</v>
+      </c>
+      <c r="D132" t="n">
+        <v>7222</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>busafsluitmodule</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>PANEL_INTERN</t>
+        </is>
+      </c>
+      <c r="C133" t="n">
+        <v>85</v>
+      </c>
+      <c r="D133" t="n">
+        <v>7222</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>netwerkmodule</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>PANEL_INTERN</t>
+        </is>
+      </c>
+      <c r="C134" t="n">
+        <v>85</v>
+      </c>
+      <c r="D134" t="n">
+        <v>7222</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>communicatiebase</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>PANEL_INTERN</t>
+        </is>
+      </c>
+      <c r="C135" t="n">
+        <v>85</v>
+      </c>
+      <c r="D135" t="n">
+        <v>7222</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>ingangsbase</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>PANEL_INTERN</t>
+        </is>
+      </c>
+      <c r="C136" t="n">
+        <v>85</v>
+      </c>
+      <c r="D136" t="n">
+        <v>7222</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>uitgangsbase</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>PANEL_INTERN</t>
+        </is>
+      </c>
+      <c r="C137" t="n">
+        <v>85</v>
+      </c>
+      <c r="D137" t="n">
+        <v>7222</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>basismodule</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>PANEL_INTERN</t>
+        </is>
+      </c>
+      <c r="C138" t="n">
+        <v>85</v>
+      </c>
+      <c r="D138" t="n">
+        <v>7222</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>aqb2005</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>METER_OPTIE_VOELER</t>
+        </is>
+      </c>
+      <c r="C139" t="n">
+        <v>90</v>
+      </c>
+      <c r="D139" t="n">
+        <v>7222</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>aqb2002</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>METER_OPTIE_VOELER</t>
+        </is>
+      </c>
+      <c r="C140" t="n">
+        <v>90</v>
+      </c>
+      <c r="D140" t="n">
+        <v>7222</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>connection set</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>METER_OPTIE_VOELER</t>
+        </is>
+      </c>
+      <c r="C141" t="n">
+        <v>90</v>
+      </c>
+      <c r="D141" t="n">
+        <v>7222</v>
       </c>
     </row>
   </sheetData>
@@ -3117,12 +3477,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G52"/>
+  <dimension ref="A1:G55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" style="9" min="1" max="1"/>
-    <col width="36" customWidth="1" style="9" min="2" max="5"/>
-    <col width="52" customWidth="1" style="9" min="6" max="6"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="5"/>
+    <col width="52" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3165,379 +3525,379 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>METING_PASSIEF</t>
         </is>
       </c>
-      <c r="B4" s="7" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>DRAK SIGK B2CA 1X2X0,8 2501 MT</t>
         </is>
       </c>
-      <c r="C4" s="7" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>DRAK SIGK CCA 1X2X0,8 2501 MT</t>
         </is>
       </c>
-      <c r="D4" s="7" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>JOBA ST.STR B2CA HCHOZ 2X1 MT</t>
         </is>
       </c>
-      <c r="E4" s="7" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>JOBA ST.STR CCA HCHOZ 2X1 MT</t>
         </is>
       </c>
-      <c r="F4" s="7" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>passive temperature sensor</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>MELDING</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>DRAK B2CA GY 2X0,8 MT</t>
         </is>
       </c>
-      <c r="C5" s="7" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>DRAK CCA GY 2X0,8 MT</t>
         </is>
       </c>
-      <c r="D5" s="7" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>JOBA ST.STR B2CA HCHOZ 2X1 MT</t>
         </is>
       </c>
-      <c r="E5" s="7" t="inlineStr">
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>JOBA ST.STR CCA HCHOZ 2X1 MT</t>
         </is>
       </c>
-      <c r="F5" s="7" t="inlineStr">
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>single volt-free contact</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>STURING_0_10V</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>RAK SIGN KAB B2CA 4X0,8 HA500</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>RAK SIGN KAB CCA 4X0,8 HA500</t>
         </is>
       </c>
-      <c r="D6" s="7" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>JOBA ST.STR B2CA HCHOZ 2X1 MT</t>
         </is>
       </c>
-      <c r="E6" s="7" t="inlineStr">
+      <c r="E6" s="3" t="inlineStr">
         <is>
           <t>JOBA ST.STR B2CA HCHOZ 2X1 MT</t>
         </is>
       </c>
-      <c r="F6" s="7" t="inlineStr">
+      <c r="F6" s="3" t="inlineStr">
         <is>
           <t>standalone AO (E-boiler sturing = 2X1!)</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>TRACING_TERUGMELDING</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>DRAK B2CA GY 2X0,8 MT</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>DRAK CCA GY 2X0,8 MT</t>
         </is>
       </c>
-      <c r="D7" s="7" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>JOBA ST.STR B2CA HCHOZ 2X1 MT</t>
         </is>
       </c>
-      <c r="E7" s="7" t="inlineStr">
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>JOBA ST.STR CCA HCHOZ 2X1 MT</t>
         </is>
       </c>
-      <c r="F7" s="7" t="n"/>
+      <c r="F7" s="3" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>METING_ACTIEF</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>DRAK SIGK B2CA 1X4X0,8 2502Q MT</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>DRAK SIGK CCA 1X4X0,8 2502Q MT</t>
         </is>
       </c>
-      <c r="D8" s="7" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>JOBA ST.STR B2CA HCHJZ 5X1 MT</t>
         </is>
       </c>
-      <c r="E8" s="7" t="inlineStr">
+      <c r="E8" s="3" t="inlineStr">
         <is>
           <t>JOBA ST.STR CCA HCHJZ 5X1 MT</t>
         </is>
       </c>
-      <c r="F8" s="7" t="inlineStr">
+      <c r="F8" s="3" t="inlineStr">
         <is>
           <t>powered sensor, feed+signal on 1 cable up to ~30VA</t>
         </is>
       </c>
     </row>
-    <row r="9" customFormat="1" s="8">
-      <c r="A9" s="7" t="inlineStr">
+    <row r="9" customFormat="1" s="7">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>METER_VOEDING_24V</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>RAK SIGN KAB B2CA 4X0,8 HA500</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>RAK SIGN KAB CCA 4X0,8 HA500</t>
         </is>
       </c>
-      <c r="D9" s="7" t="inlineStr">
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>JOBA ST.STR B2CA HCHJZ 5X1 MT</t>
         </is>
       </c>
-      <c r="E9" s="7" t="inlineStr">
+      <c r="E9" s="3" t="inlineStr">
         <is>
           <t>JOBA ST.STR CCA HCHJZ 5X1 MT</t>
         </is>
       </c>
-      <c r="F9" s="7" t="inlineStr">
+      <c r="F9" s="3" t="inlineStr">
         <is>
           <t>separate feed cable energy meter — CCA per Boerhaave (3X1), B2CA per Duitslandlaan (5X1)</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="inlineStr">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>REGELAFSLUITER_0_10V</t>
         </is>
       </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>RAK SIGN KAB B2CA 4X0,8 HA500</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>RAK SIGN KAB CCA 4X0,8 HA500</t>
         </is>
       </c>
-      <c r="D10" s="7" t="inlineStr">
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>JOBA ST.STR B2CA HCHJZ 5X1 MT</t>
         </is>
       </c>
-      <c r="E10" s="7" t="inlineStr">
+      <c r="E10" s="3" t="inlineStr">
         <is>
           <t>JOBA ST.STR CCA HCHJZ 5X1 MT</t>
         </is>
       </c>
-      <c r="F10" s="7" t="n"/>
+      <c r="F10" s="3" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>VRIJGAVE_STORING</t>
         </is>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>DRAK SIGK B2CA 1X4X0,8 2502Q MT</t>
         </is>
       </c>
-      <c r="C11" s="7" t="inlineStr">
+      <c r="C11" s="3" t="inlineStr">
         <is>
           <t>DRAK SIGK CCA 1X4X0,8 2502Q MT</t>
         </is>
       </c>
-      <c r="D11" s="7" t="inlineStr">
+      <c r="D11" s="3" t="inlineStr">
         <is>
           <t>JOBA ST.STR B2CA HCHJZ 5X1 MT</t>
         </is>
       </c>
-      <c r="E11" s="7" t="inlineStr">
+      <c r="E11" s="3" t="inlineStr">
         <is>
           <t>JOBA ST.STR CCA HCHJZ 5X1 MT</t>
         </is>
       </c>
-      <c r="F11" s="7" t="inlineStr">
+      <c r="F11" s="3" t="inlineStr">
         <is>
           <t>E-boiler enable/fault</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="inlineStr">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>BEDRIJF_STORING</t>
         </is>
       </c>
-      <c r="B12" s="7" t="inlineStr">
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>RAK SIGN KAB B2CA 4X0,8 HA500</t>
         </is>
       </c>
-      <c r="C12" s="7" t="inlineStr">
+      <c r="C12" s="3" t="inlineStr">
         <is>
           <t>RAK SIGN KAB CCA 4X0,8 HA500</t>
         </is>
       </c>
-      <c r="D12" s="7" t="inlineStr">
+      <c r="D12" s="3" t="inlineStr">
         <is>
           <t>JOBA ST.STR B2CA HCHJZ 5X1 MT</t>
         </is>
       </c>
-      <c r="E12" s="7" t="inlineStr">
+      <c r="E12" s="3" t="inlineStr">
         <is>
           <t>JOBA ST.STR CCA HCHJZ 5X1 MT</t>
         </is>
       </c>
-      <c r="F12" s="7" t="n"/>
+      <c r="F12" s="3" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="inlineStr">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>KLEP_STURING_MELDING</t>
         </is>
       </c>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>DRAK B2CA GY 6X0,8 MT</t>
         </is>
       </c>
-      <c r="C13" s="7" t="inlineStr">
+      <c r="C13" s="3" t="inlineStr">
         <is>
           <t>DRAK CCA GY 6X0,8 MT</t>
         </is>
       </c>
-      <c r="D13" s="7" t="inlineStr">
+      <c r="D13" s="3" t="inlineStr">
         <is>
           <t>JOBA STSTR B2CA HCHJZ 7X1 MT</t>
         </is>
       </c>
-      <c r="E13" s="7" t="inlineStr">
+      <c r="E13" s="3" t="inlineStr">
         <is>
           <t>JOBA STSTR CCA HCHJZ 7X1 MT</t>
         </is>
       </c>
-      <c r="F13" s="7" t="inlineStr">
+      <c r="F13" s="3" t="inlineStr">
         <is>
           <t>isolation valve control + feedback</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="inlineStr">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>KLEP_OD</t>
         </is>
       </c>
-      <c r="B14" s="7" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
         <is>
           <t>DRAK B2CA GY 8X0,8 MT</t>
         </is>
       </c>
-      <c r="C14" s="7" t="inlineStr">
+      <c r="C14" s="3" t="inlineStr">
         <is>
           <t>DRAK CCA GY 8X0,8 MT</t>
         </is>
       </c>
-      <c r="D14" s="7" t="inlineStr">
+      <c r="D14" s="3" t="inlineStr">
         <is>
           <t>JOBA ST.STR B2CA HCHJZ 7X1 MT</t>
         </is>
       </c>
-      <c r="E14" s="7" t="inlineStr">
+      <c r="E14" s="3" t="inlineStr">
         <is>
           <t>JOBA ST.STR CCA HCHJZ 7X1 MT</t>
         </is>
       </c>
-      <c r="F14" s="7" t="inlineStr">
+      <c r="F14" s="3" t="inlineStr">
         <is>
           <t>open/close + feedback(s)</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="inlineStr">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>BRANDKLEP</t>
         </is>
       </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>RAK SIGN KAB B2CA 4X0,8 HA500</t>
         </is>
       </c>
-      <c r="C15" s="7" t="inlineStr">
+      <c r="C15" s="3" t="inlineStr">
         <is>
           <t>RAK SIGN KAB CCA 4X0,8 HA500</t>
         </is>
       </c>
-      <c r="D15" s="7" t="inlineStr">
+      <c r="D15" s="3" t="inlineStr">
         <is>
           <t>JOBA ST.STR B2CA HCHOZ 2X1 MT</t>
         </is>
       </c>
-      <c r="E15" s="7" t="inlineStr">
+      <c r="E15" s="3" t="inlineStr">
         <is>
           <t>JOBA ST.STR CCA HCHOZ 2X1 MT</t>
         </is>
       </c>
-      <c r="F15" s="7" t="inlineStr">
+      <c r="F15" s="3" t="inlineStr">
         <is>
           <t>one cable PER damper (112)</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="7" t="inlineStr">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>MELDINGEN_GROOT</t>
         </is>
@@ -3552,55 +3912,55 @@
           <t>DRAK SIGK AFG CCA 4X2X0,8 MT</t>
         </is>
       </c>
-      <c r="D16" s="7" t="inlineStr">
+      <c r="D16" s="3" t="inlineStr">
         <is>
           <t>JOBA HCH-JZ 12X1 B2CA MT</t>
         </is>
       </c>
-      <c r="E16" s="7" t="inlineStr">
+      <c r="E16" s="3" t="inlineStr">
         <is>
           <t>JOBA HCH-JZ 12X1 B2CA MT</t>
         </is>
       </c>
-      <c r="F16" s="7" t="inlineStr">
+      <c r="F16" s="3" t="inlineStr">
         <is>
           <t>WP meldingen, fan 'diverse functions'</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="7" t="inlineStr">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>EC_VENTILATOR</t>
         </is>
       </c>
-      <c r="B17" s="7" t="inlineStr">
+      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>DRAK SIGK AFG B2CA 3X2X0,8 MT</t>
         </is>
       </c>
-      <c r="C17" s="7" t="inlineStr">
+      <c r="C17" s="3" t="inlineStr">
         <is>
           <t>DRAK SIGK AFG CCA 3X2X0,8 MT</t>
         </is>
       </c>
-      <c r="D17" s="7" t="inlineStr">
+      <c r="D17" s="3" t="inlineStr">
         <is>
           <t>JOBA ST.STR B2CA HCHJZ 7X1 MT</t>
         </is>
       </c>
-      <c r="E17" s="7" t="inlineStr">
+      <c r="E17" s="3" t="inlineStr">
         <is>
           <t>JOBA ST.STR B2CA HCHJZ 7X1 MT</t>
         </is>
       </c>
-      <c r="F17" s="7" t="inlineStr">
+      <c r="F17" s="3" t="inlineStr">
         <is>
           <t>run/fault/control</t>
         </is>
       </c>
     </row>
-    <row r="18" s="9">
+    <row r="18">
       <c r="A18" t="inlineStr">
         <is>
           <t>SMOORAFSLUITER</t>
@@ -3660,7 +4020,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>boiler feed (dict: Ketel 1/2/3/4 voeding 3g1,5). Encoded as 3G2,5 to match validated project practice on 230V pumps; dict spec 3g1,5 is minimum. Ask Rick.</t>
+          <t>boiler feed (dict: Ketel 1/2/3/4 voeding 3g2,5). Encoded as 3G2,5 to match validated project practice on 230V pumps; dict spec 3g2,5 is minimum. Ask Rick.</t>
         </is>
       </c>
     </row>
@@ -3672,22 +4032,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>DRAK HULT B2CA 5G1,5 HA500</t>
+          <t>DRAK HULT B2CA 5G2,5 HA500</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>DRAK HULT CCA 5G1,5 HA500</t>
+          <t>DRAK HULT CCA 5G2,5 HA500</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>DRAK HULT B2CA 5G1,5 MT</t>
+          <t>DRAK HULT B2CA 5G2,5 MT</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>DRAK HULT CCA 5G1,5 MT</t>
+          <t>DRAK HULT CCA 5G2,5 MT</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -3712,12 +4072,12 @@
           <t>DRAK CCA GY 6X0,8 MT</t>
         </is>
       </c>
-      <c r="D21" s="7" t="inlineStr">
+      <c r="D21" s="3" t="inlineStr">
         <is>
           <t>JOBA ST.STR B2CA HCHJZ 7X1 MT</t>
         </is>
       </c>
-      <c r="E21" s="7" t="inlineStr">
+      <c r="E21" s="3" t="inlineStr">
         <is>
           <t>JOBA ST.STR CCA HCHJZ 7X1 MT</t>
         </is>
@@ -3736,22 +4096,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>DRAK HULT B2CA 3G1,5 HA500</t>
+          <t>DRAK HULT B2CA 3G2,5 HA500</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>DRAK HULT CCA 3G1,5 HA500</t>
+          <t>DRAK HULT CCA 3G2,5 HA500</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>DRAK HULT B2CA 3G1,5 MT</t>
+          <t>DRAK HULT B2CA 3G2,5 MT</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>DRAK HULT CCA 3G1,5 MT</t>
+          <t>DRAK HULT CCA 3G2,5 MT</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -3776,12 +4136,12 @@
           <t>DRAK SIGK AFG CCA 3X2X0,8 MT</t>
         </is>
       </c>
-      <c r="D23" s="7" t="inlineStr">
+      <c r="D23" s="3" t="inlineStr">
         <is>
           <t>JOBA ST.STR B2CA HCHJZ 7X1 MT</t>
         </is>
       </c>
-      <c r="E23" s="7" t="inlineStr">
+      <c r="E23" s="3" t="inlineStr">
         <is>
           <t>JOBA ST.STR B2CA HCHJZ 7X1 MT</t>
         </is>
@@ -3808,12 +4168,12 @@
           <t>DRAK CCA GY 4X0,8 MT</t>
         </is>
       </c>
-      <c r="D24" s="7" t="inlineStr">
+      <c r="D24" s="3" t="inlineStr">
         <is>
           <t>JOBA ST.STR B2CA HCHJZ 5X1 MT</t>
         </is>
       </c>
-      <c r="E24" s="7" t="inlineStr">
+      <c r="E24" s="3" t="inlineStr">
         <is>
           <t>JOBA ST.STR CCA HCHJZ 5X1 MT</t>
         </is>
@@ -3840,12 +4200,12 @@
           <t>DRAK CCA GY 4X0,8 MT</t>
         </is>
       </c>
-      <c r="D25" s="7" t="inlineStr">
+      <c r="D25" s="3" t="inlineStr">
         <is>
           <t>JOBA ST.STR B2CA HCHJZ 5X1 MT</t>
         </is>
       </c>
-      <c r="E25" s="7" t="inlineStr">
+      <c r="E25" s="3" t="inlineStr">
         <is>
           <t>JOBA ST.STR CCA HCHJZ 5X1 MT</t>
         </is>
@@ -3872,12 +4232,12 @@
           <t>DRAK CCA GY 4X0,8 MT</t>
         </is>
       </c>
-      <c r="D26" s="7" t="inlineStr">
+      <c r="D26" s="3" t="inlineStr">
         <is>
           <t>JOBA ST.STR B2CA HCHJZ 5X1 MT</t>
         </is>
       </c>
-      <c r="E26" s="7" t="inlineStr">
+      <c r="E26" s="3" t="inlineStr">
         <is>
           <t>JOBA ST.STR CCA HCHJZ 5X1 MT</t>
         </is>
@@ -3894,22 +4254,22 @@
           <t>STOOMBEVOCHTIGER_STURING</t>
         </is>
       </c>
-      <c r="B27" s="7" t="inlineStr">
+      <c r="B27" s="3" t="inlineStr">
         <is>
           <t>DRAK SIGK B2CA 1X4X0,8 2502Q MT</t>
         </is>
       </c>
-      <c r="C27" s="7" t="inlineStr">
+      <c r="C27" s="3" t="inlineStr">
         <is>
           <t>DRAK SIGK CCA 1X4X0,8 2502Q MT</t>
         </is>
       </c>
-      <c r="D27" s="7" t="inlineStr">
+      <c r="D27" s="3" t="inlineStr">
         <is>
           <t>JOBA ST.STR B2CA HCHJZ 5X1 MT</t>
         </is>
       </c>
-      <c r="E27" s="7" t="inlineStr">
+      <c r="E27" s="3" t="inlineStr">
         <is>
           <t>JOBA ST.STR B2CA HCHJZ 5X1 MT</t>
         </is>
@@ -3936,12 +4296,12 @@
           <t>DRAK CCA GY 4X0,8 MT</t>
         </is>
       </c>
-      <c r="D28" s="7" t="inlineStr">
+      <c r="D28" s="3" t="inlineStr">
         <is>
           <t>JOBA ST.STR B2CA HCHJZ 5X1 MT</t>
         </is>
       </c>
-      <c r="E28" s="7" t="inlineStr">
+      <c r="E28" s="3" t="inlineStr">
         <is>
           <t>JOBA ST.STR CCA HCHJZ 5X1 MT</t>
         </is>
@@ -3968,12 +4328,12 @@
           <t>DRAK CCA GY 4X0,8 MT</t>
         </is>
       </c>
-      <c r="D29" s="7" t="inlineStr">
+      <c r="D29" s="3" t="inlineStr">
         <is>
           <t>JOBA ST.STR B2CA HCHJZ 5X1 MT</t>
         </is>
       </c>
-      <c r="E29" s="7" t="inlineStr">
+      <c r="E29" s="3" t="inlineStr">
         <is>
           <t>JOBA ST.STR CCA HCHJZ 5X1 MT</t>
         </is>
@@ -4022,22 +4382,22 @@
           <t>VENTILATOR_STURING</t>
         </is>
       </c>
-      <c r="B31" s="7" t="inlineStr">
+      <c r="B31" s="3" t="inlineStr">
         <is>
           <t>DRAK SIGK B2CA 1X4X0,8 2502Q MT</t>
         </is>
       </c>
-      <c r="C31" s="7" t="inlineStr">
+      <c r="C31" s="3" t="inlineStr">
         <is>
           <t>DRAK SIGK CCA 1X4X0,8 2502Q MT</t>
         </is>
       </c>
-      <c r="D31" s="7" t="inlineStr">
+      <c r="D31" s="3" t="inlineStr">
         <is>
           <t>JOBA ST.STR B2CA HCHJZ 5X1 MT</t>
         </is>
       </c>
-      <c r="E31" s="7" t="inlineStr">
+      <c r="E31" s="3" t="inlineStr">
         <is>
           <t>JOBA ST.STR CCA HCHJZ 5X1 MT</t>
         </is>
@@ -4096,12 +4456,12 @@
           <t>DRAK CCA GY 4X0,8 MT</t>
         </is>
       </c>
-      <c r="D33" s="7" t="inlineStr">
+      <c r="D33" s="3" t="inlineStr">
         <is>
           <t>JOBA ST.STR B2CA HCHJZ 5X1 MT</t>
         </is>
       </c>
-      <c r="E33" s="7" t="inlineStr">
+      <c r="E33" s="3" t="inlineStr">
         <is>
           <t>JOBA ST.STR CCA HCHJZ 5X1 MT</t>
         </is>
@@ -4128,12 +4488,12 @@
           <t>DRAK CCA GY 4X0,8 MT</t>
         </is>
       </c>
-      <c r="D34" s="7" t="inlineStr">
+      <c r="D34" s="3" t="inlineStr">
         <is>
           <t>JOBA ST.STR B2CA HCHJZ 5X1 MT</t>
         </is>
       </c>
-      <c r="E34" s="7" t="inlineStr">
+      <c r="E34" s="3" t="inlineStr">
         <is>
           <t>JOBA ST.STR CCA HCHJZ 5X1 MT</t>
         </is>
@@ -4160,12 +4520,12 @@
           <t>DRAK CCA GY 6X0,8 MT</t>
         </is>
       </c>
-      <c r="D35" s="7" t="inlineStr">
+      <c r="D35" s="3" t="inlineStr">
         <is>
           <t>JOBA ST.STR B2CA HCHJZ 12X1 MT</t>
         </is>
       </c>
-      <c r="E35" s="7" t="inlineStr">
+      <c r="E35" s="3" t="inlineStr">
         <is>
           <t>JOBA ST.STR CCA HCHJZ 10X1 MT</t>
         </is>
@@ -4192,12 +4552,12 @@
           <t>DRAK CCA GY 4X0,8 MT</t>
         </is>
       </c>
-      <c r="D36" s="7" t="inlineStr">
+      <c r="D36" s="3" t="inlineStr">
         <is>
           <t>JOBA ST.STR B2CA HCHJZ 5X1 MT</t>
         </is>
       </c>
-      <c r="E36" s="7" t="inlineStr">
+      <c r="E36" s="3" t="inlineStr">
         <is>
           <t>JOBA ST.STR B2CA HCHJZ 5X1 MT</t>
         </is>
@@ -4224,12 +4584,12 @@
           <t>DRAK CCA GY 4X0,8 MT</t>
         </is>
       </c>
-      <c r="D37" s="7" t="inlineStr">
+      <c r="D37" s="3" t="inlineStr">
         <is>
           <t>JOBA ST.STR B2CA HCHJZ 5X1 MT</t>
         </is>
       </c>
-      <c r="E37" s="7" t="inlineStr">
+      <c r="E37" s="3" t="inlineStr">
         <is>
           <t>JOBA ST.STR CCA HCHJZ 5X1 MT</t>
         </is>
@@ -4320,12 +4680,12 @@
           <t>DRAK SIGK CCA 1X4X0,8 2501 MT</t>
         </is>
       </c>
-      <c r="D40" s="7" t="inlineStr">
+      <c r="D40" s="3" t="inlineStr">
         <is>
           <t>JOBA ST.STR B2CA HCHJZ 5X1 MT</t>
         </is>
       </c>
-      <c r="E40" s="7" t="inlineStr">
+      <c r="E40" s="3" t="inlineStr">
         <is>
           <t>JOBA ST.STR B2CA HCHJZ 5X1 MT</t>
         </is>
@@ -4342,22 +4702,22 @@
           <t>GASDETECTIE</t>
         </is>
       </c>
-      <c r="B41" s="7" t="inlineStr">
+      <c r="B41" s="3" t="inlineStr">
         <is>
           <t>DRAK SIGK B2CA 1X4X0,8 2502Q MT</t>
         </is>
       </c>
-      <c r="C41" s="7" t="inlineStr">
+      <c r="C41" s="3" t="inlineStr">
         <is>
           <t>DRAK SIGK CCA 1X4X0,8 2502Q MT</t>
         </is>
       </c>
-      <c r="D41" s="7" t="inlineStr">
+      <c r="D41" s="3" t="inlineStr">
         <is>
           <t>JOBA ST.STR B2CA HCHJZ 5X1 MT</t>
         </is>
       </c>
-      <c r="E41" s="7" t="inlineStr">
+      <c r="E41" s="3" t="inlineStr">
         <is>
           <t>JOBA ST.STR CCA HCHJZ 5X1 MT</t>
         </is>
@@ -4416,12 +4776,12 @@
           <t>DRAK CCA GY 4X0,8 MT</t>
         </is>
       </c>
-      <c r="D43" s="7" t="inlineStr">
+      <c r="D43" s="3" t="inlineStr">
         <is>
           <t>JOBA ST.STR B2CA HCHJZ 5X1 MT</t>
         </is>
       </c>
-      <c r="E43" s="7" t="inlineStr">
+      <c r="E43" s="3" t="inlineStr">
         <is>
           <t>JOBA ST.STR CCA HCHJZ 5X1 MT</t>
         </is>
@@ -4432,28 +4792,28 @@
         </is>
       </c>
     </row>
-    <row r="44" s="9">
+    <row r="44">
       <c r="A44" t="inlineStr">
         <is>
           <t>WEERSTATION_BUS</t>
         </is>
       </c>
-      <c r="B44" s="10" t="inlineStr">
+      <c r="B44" s="8" t="inlineStr">
         <is>
           <t>BMS Cable 2x2x24AWG - R1319 - B2ca s1,d0,a1 Violet HA500</t>
         </is>
       </c>
-      <c r="C44" s="10" t="inlineStr">
+      <c r="C44" s="8" t="inlineStr">
         <is>
           <t>BMS Cable 2x2x24AWG - R1319 -  B2ca s1,d0,a1 Violet HA500</t>
         </is>
       </c>
-      <c r="D44" s="10" t="inlineStr">
+      <c r="D44" s="8" t="inlineStr">
         <is>
           <t>BMS Cable 2x2x24AWG - R1319 - B2ca s1,d0,a1 Violet HA500</t>
         </is>
       </c>
-      <c r="E44" s="10" t="inlineStr">
+      <c r="E44" s="8" t="inlineStr">
         <is>
           <t>BMS Cable 2x2x24AWG - R1319 -  CCA s1,d0,a1 Violet HA500</t>
         </is>
@@ -4477,22 +4837,22 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>DRAK HULT B2CA 5G1,5 HA500</t>
+          <t>DRAK HULT B2CA 5G2,5 HA500</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>DRAK HULT CCA 5G1,5 HA500</t>
+          <t>DRAK HULT CCA 5G2,5 HA500</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>DRAK HULT B2CA 5G1,5 MT</t>
+          <t>DRAK HULT B2CA 5G2,5 MT</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>DRAK HULT CCA 5G1,5 MT</t>
+          <t>DRAK HULT CCA 5G2,5 MT</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -4517,12 +4877,12 @@
           <t>DRAK CCA GY 4X0,8 MT</t>
         </is>
       </c>
-      <c r="D46" s="7" t="inlineStr">
+      <c r="D46" s="3" t="inlineStr">
         <is>
           <t>JOBA ST.STR B2CA HCHJZ 5X1 MT</t>
         </is>
       </c>
-      <c r="E46" s="7" t="inlineStr">
+      <c r="E46" s="3" t="inlineStr">
         <is>
           <t>JOBA ST.STR CCA HCHJZ 5X1 MT</t>
         </is>
@@ -4549,12 +4909,12 @@
           <t>DRAK CCA GY 4X0,8 MT</t>
         </is>
       </c>
-      <c r="D47" s="7" t="inlineStr">
+      <c r="D47" s="3" t="inlineStr">
         <is>
           <t>JOBA ST.STR B2CA HCHJZ 5X1 MT</t>
         </is>
       </c>
-      <c r="E47" s="7" t="inlineStr">
+      <c r="E47" s="3" t="inlineStr">
         <is>
           <t>JOBA ST.STR CCA HCHJZ 5X1 MT</t>
         </is>
@@ -4571,22 +4931,22 @@
           <t>DRUKOPNEMER_PASSIEF</t>
         </is>
       </c>
-      <c r="B48" s="7" t="inlineStr">
+      <c r="B48" s="3" t="inlineStr">
         <is>
           <t>DRAK SIGK B2CA 1X4X0,8 2502Q MT</t>
         </is>
       </c>
-      <c r="C48" s="7" t="inlineStr">
+      <c r="C48" s="3" t="inlineStr">
         <is>
           <t>DRAK SIGK CCA 1X4X0,8 2502Q MT</t>
         </is>
       </c>
-      <c r="D48" s="7" t="inlineStr">
+      <c r="D48" s="3" t="inlineStr">
         <is>
           <t>JOBA ST.STR B2CA HCHJZ 5X1 MT</t>
         </is>
       </c>
-      <c r="E48" s="7" t="inlineStr">
+      <c r="E48" s="3" t="inlineStr">
         <is>
           <t>JOBA ST.STR B2CA HCHJZ 5X1 MT</t>
         </is>
@@ -4613,12 +4973,12 @@
           <t>DRAK CCA GY 6X0,8 MT</t>
         </is>
       </c>
-      <c r="D49" s="7" t="inlineStr">
+      <c r="D49" s="3" t="inlineStr">
         <is>
           <t>JOBA ST.STR B2CA HCHJZ 7X1 MT</t>
         </is>
       </c>
-      <c r="E49" s="7" t="inlineStr">
+      <c r="E49" s="3" t="inlineStr">
         <is>
           <t>JOBA ST.STR CCA HCHJZ 7X1 MT</t>
         </is>
@@ -4629,28 +4989,28 @@
         </is>
       </c>
     </row>
-    <row r="50" s="9">
+    <row r="50">
       <c r="A50" t="inlineStr">
         <is>
           <t>KOELMACHINE_MODBUS</t>
         </is>
       </c>
-      <c r="B50" s="10" t="inlineStr">
+      <c r="B50" s="8" t="inlineStr">
         <is>
           <t>BMS Cable 2x2x24AWG - R1319 - B2ca s1,d0,a1 Violet HA500</t>
         </is>
       </c>
-      <c r="C50" s="10" t="inlineStr">
+      <c r="C50" s="8" t="inlineStr">
         <is>
           <t>BMS Cable 2x2x24AWG - R1319 - B2ca s1,d0,a1 Violet HA500</t>
         </is>
       </c>
-      <c r="D50" s="10" t="inlineStr">
+      <c r="D50" s="8" t="inlineStr">
         <is>
           <t>BMS Cable 2x2x24AWG - R1319 - B2ca s1,d0,a1 Violet HA500</t>
         </is>
       </c>
-      <c r="E50" s="10" t="inlineStr">
+      <c r="E50" s="8" t="inlineStr">
         <is>
           <t>BMS Cable 2x2x24AWG - R1319 -  CCA s1,d0,a1 Violet HA500</t>
         </is>
@@ -4677,12 +5037,12 @@
           <t>DRAK CCA GY 4X0,8 MT</t>
         </is>
       </c>
-      <c r="D51" s="7" t="inlineStr">
+      <c r="D51" s="3" t="inlineStr">
         <is>
           <t>JOBA ST.STR B2CA HCHJZ 5X1 MT</t>
         </is>
       </c>
-      <c r="E51" s="7" t="inlineStr">
+      <c r="E51" s="3" t="inlineStr">
         <is>
           <t>JOBA ST.STR B2CA HCHJZ 5X1 MT</t>
         </is>
@@ -4709,12 +5069,12 @@
           <t>DRAK SIGK CCA 1X4X0,8 2502Q MT</t>
         </is>
       </c>
-      <c r="D52" s="7" t="inlineStr">
+      <c r="D52" s="3" t="inlineStr">
         <is>
           <t>JOBA ST.STR B2CA HCHJZ 5X1 MT</t>
         </is>
       </c>
-      <c r="E52" s="7" t="inlineStr">
+      <c r="E52" s="3" t="inlineStr">
         <is>
           <t>JOBA ST.STR CCA HCHJZ 5X1 MT</t>
         </is>
@@ -4722,6 +5082,87 @@
       <c r="F52" t="inlineStr">
         <is>
           <t>B2CA HA500	bus-connected temp sensor, no AI by design; B2CA value from 2195-06 manual — UNCONFIRMED</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" customFormat="1" s="10">
+      <c r="A53" s="10" t="inlineStr">
+        <is>
+          <t>KLEP_OD_ZONDER_TERUGMELDING</t>
+        </is>
+      </c>
+      <c r="B53" s="10" t="inlineStr">
+        <is>
+          <t>DRAK B2CA GY 4X0,8 MT</t>
+        </is>
+      </c>
+      <c r="C53" s="10" t="inlineStr">
+        <is>
+          <t>DRAK CCA GY 4X0,8 MT</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="10" t="inlineStr">
+        <is>
+          <t>POMP_2_SIGNALEN</t>
+        </is>
+      </c>
+      <c r="B54" s="10" t="inlineStr">
+        <is>
+          <t>1x4x0,8</t>
+        </is>
+      </c>
+      <c r="C54" s="10" t="inlineStr">
+        <is>
+          <t>1x4x0,8</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>1x4x0,8</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>1x4x0,8</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>pomp met 2 signalen (vrijgave/storing). Rick 2026-08-18 + CCA dictionary. Dictionary value is family-agnostic, so identical in all four columns. Pump-specific: dict gives a 3-signal KETEL 1x4x0,8 and a 2-signal VENTILATOR 2x2x0,8, so do NOT generalise the count rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="10" t="inlineStr">
+        <is>
+          <t>POMP_3_SIGNALEN</t>
+        </is>
+      </c>
+      <c r="B55" s="10" t="inlineStr">
+        <is>
+          <t>3x2x0,8</t>
+        </is>
+      </c>
+      <c r="C55" s="10" t="inlineStr">
+        <is>
+          <t>3x2x0,8</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>3x2x0,8</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>3x2x0,8</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>pomp met 3 signalen (vrijgave/storing/sturing). Rick 2026-08-18 + CCA dictionary. Family-agnostic. 7222 manual writes this as DRAK KAB AFG B2CA 3X2X0,8 MT (x32).</t>
         </is>
       </c>
     </row>
@@ -4739,10 +5180,10 @@
   <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" style="9" min="1" max="1"/>
-    <col width="46" customWidth="1" style="9" min="2" max="3"/>
-    <col width="6" customWidth="1" style="9" min="4" max="4"/>
-    <col width="26" customWidth="1" style="9" min="5" max="5"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="2" max="3"/>
+    <col width="6" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4800,98 +5241,98 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>230V_1F</t>
         </is>
       </c>
-      <c r="B4" s="7" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>DRAK HULT CCA 3G2,5 HA500</t>
         </is>
       </c>
-      <c r="C4" s="7" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>DRAK HULT B2CA 3G2,5 MT</t>
         </is>
       </c>
-      <c r="D4" s="7" t="n">
+      <c r="D4" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="E4" s="7" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>{kw}kW/{a}A/230V</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>400V_3F_zonder_N</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>DRAK HULT CCA 4X2,5 MT</t>
         </is>
       </c>
-      <c r="C5" s="7" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>DRAK HULT B2CA 4G2,5 MT</t>
         </is>
       </c>
-      <c r="D5" s="7" t="n">
+      <c r="D5" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="E5" s="7" t="inlineStr">
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>{kw}kW/{a}A/400V</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>400V_3F_met_N</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>DRAK HULT CCA 5G2,5 MT</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>DRAK HULT B2CA 5G2,5 MT</t>
         </is>
       </c>
-      <c r="D6" s="7" t="n">
+      <c r="D6" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="E6" s="7" t="inlineStr">
+      <c r="E6" s="3" t="inlineStr">
         <is>
           <t>{kw}kW/{a}A/400V</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>TRACING</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>DRAK HULT CCA 5G2,5 MT</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>DRAK HULT B2CA 3G2,5 MT</t>
         </is>
       </c>
-      <c r="D7" s="7" t="n"/>
-      <c r="E7" s="7" t="n"/>
+      <c r="D7" s="3" t="n"/>
+      <c r="E7" s="3" t="n"/>
       <c r="G7" t="n">
         <v>1</v>
       </c>
@@ -4902,42 +5343,42 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>DERDEN_RK</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>Kabel levering derde totaan RK, aansluiten kastzijde Erco</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>Kabel levering derde totaan RK, aansluiten kastzijde Erco</t>
         </is>
       </c>
-      <c r="D8" s="7" t="n"/>
-      <c r="E8" s="7" t="n"/>
+      <c r="D8" s="3" t="n"/>
+      <c r="E8" s="3" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>DERDEN_TOESTEL</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>Werkzaamheden derden</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>Werkzaamheden derden</t>
         </is>
       </c>
-      <c r="D9" s="7" t="n"/>
-      <c r="E9" s="7" t="n"/>
+      <c r="D9" s="3" t="n"/>
+      <c r="E9" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4953,10 +5394,10 @@
   <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" style="9" min="1" max="1"/>
-    <col width="56" customWidth="1" style="9" min="2" max="2"/>
-    <col width="14" customWidth="1" style="9" min="3" max="3"/>
-    <col width="56" customWidth="1" style="9" min="4" max="4"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="56" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="56" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4989,128 +5430,128 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>MODBUS_RTU</t>
         </is>
       </c>
-      <c r="B4" s="7" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>BMS Cable 2x2x24AWG - R1319 - B2ca s1,d0,a1 Violet HA500</t>
         </is>
       </c>
-      <c r="C4" s="7" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>doorlussen</t>
         </is>
       </c>
-      <c r="D4" s="7" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>1st device: location; 2nd+: 'doorlussen' (lowercase)</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>MODBUS_IP_VELD</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>BMS Cable 2x2x24AWG - R1319 - B2ca s1,d0,a1 Violet HA500</t>
         </is>
       </c>
-      <c r="C5" s="7" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>geen</t>
         </is>
       </c>
-      <c r="D5" s="7" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>Modbus-IP field device = BMS cable, NO UTP (Duitslandlaan Korex)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>BACNET_IP</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>COMM U/UTP CAT6 CS34ZB HA305</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>geen</t>
         </is>
       </c>
-      <c r="D6" s="7" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>one cable per device, no daisy-chain (112)</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>TOUCHPANEL_IP</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>GGM C6U4PFROHT3 GGM U/UTP6 LSZH 305M</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>geen</t>
         </is>
       </c>
-      <c r="D7" s="7" t="n"/>
+      <c r="D7" s="3" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>RK_ONDERLING</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>COMM U/UTP CAT6 CS34ZC HA305</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>geen</t>
         </is>
       </c>
-      <c r="D8" s="7" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>or CS34ZB, depending on the room-control system</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>MBUS_DERDEN</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>Kabel levering derde, enkelzijdig aansluiten op regelkast Erco</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>geen</t>
         </is>
       </c>
-      <c r="D9" s="7" t="n"/>
+      <c r="D9" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5126,8 +5567,8 @@
   <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" style="9" min="1" max="1"/>
-    <col width="70" customWidth="1" style="9" min="2" max="2"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="70" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5150,84 +5591,84 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>AANSLUITSNOER</t>
         </is>
       </c>
-      <c r="B4" s="7" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>Via aansluitsnoer van 2 meter op meter</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>BRANDMELDING</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>Kabel levering derde totaan RK, aansluiten kastzijde Erco</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>NAREGEL_UNIT_DERDE</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>Kabel levering derde, aanbrengen werkzaamheden Erco</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>TOT_DERDEN</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Totaal voedingen derden aansluiten</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>TOT_WS</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>Totaal aantal werkschakelaars van maximaal 63A</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>ONDERSTATION</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>Onderstation algemeen</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="inlineStr">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>VOEDINGEN</t>
         </is>
       </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>Voedingen</t>
         </is>
@@ -5283,9 +5724,9 @@
   <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="36" customWidth="1" style="9" min="1" max="1"/>
-    <col width="14" customWidth="1" style="9" min="2" max="2"/>
-    <col width="20" customWidth="1" style="9" min="3" max="3"/>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>